<commit_message>
fuseki reconfiguration to include SHACL service. Light modelling development.
</commit_message>
<xml_diff>
--- a/src/models/serialisation_templates.xlsx
+++ b/src/models/serialisation_templates.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="DMCAR" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="67">
   <si>
     <t xml:space="preserve">Namespace</t>
   </si>
@@ -156,6 +156,9 @@
     <t xml:space="preserve">SourceAttribute</t>
   </si>
   <si>
+    <t xml:space="preserve">TargetInstance</t>
+  </si>
+  <si>
     <t xml:space="preserve">TargetNamespace</t>
   </si>
   <si>
@@ -169,6 +172,39 @@
   </si>
   <si>
     <t xml:space="preserve">Translation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMCARSchema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Triple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#Namespace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#Domain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#DomainEvent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#DomainParticipant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#Attribute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#Class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.tkltd.org/ontologies/datamodel#Relationship</t>
   </si>
   <si>
     <t xml:space="preserve">Project</t>
@@ -196,7 +232,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -236,6 +272,35 @@
     </font>
     <font>
       <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -337,7 +402,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -374,11 +439,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -391,6 +472,64 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA23EFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF79FC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF8000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFBF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF333333"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -460,7 +599,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AM1"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.91"/>
@@ -633,20 +772,26 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="15.47265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M158"/>
+  <sheetFormatPr defaultColWidth="15.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="4" style="0" width="22.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="22.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="33.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="9" width="22.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="34.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="50.48"/>
   </cols>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -661,23 +806,965 @@
       <c r="G1" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" s="6" t="s">
         <v>48</v>
       </c>
+      <c r="M1" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F2" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" s="12"/>
+      <c r="J2" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L2" s="13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G4" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" s="12"/>
+      <c r="J5" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G6" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G7" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" s="12"/>
+      <c r="J8" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G9" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G10" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" s="12"/>
+      <c r="J11" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K11" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G12" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G13" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H14" s="12"/>
+      <c r="J14" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K14" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G15" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G16" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H17" s="12"/>
+      <c r="J17" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K17" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G18" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G19" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G20" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="12"/>
+      <c r="J20" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K20" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L20" s="13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G21" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G22" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" s="12"/>
+      <c r="J23" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K23" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G24" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G25" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G26" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H26" s="12"/>
+      <c r="J26" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K26" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G27" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G28" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H29" s="0"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H32" s="12"/>
+      <c r="J32" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K32" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L32" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G33" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G34" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H35" s="12"/>
+      <c r="J35" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K35" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G36" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G37" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H38" s="12"/>
+      <c r="J38" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K38" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G39" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G40" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="12"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="12"/>
+      <c r="M41" s="12"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G42" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H42" s="12"/>
+      <c r="J42" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K42" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L42" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G43" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G44" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G45" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H45" s="12"/>
+      <c r="J45" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K45" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G46" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G47" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G48" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H48" s="12"/>
+      <c r="J48" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K48" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G49" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G50" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G51" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H51" s="12"/>
+      <c r="J51" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K51" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L51" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G52" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G53" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G54" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H54" s="12"/>
+      <c r="J54" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K54" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G55" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G56" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G57" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H57" s="12"/>
+      <c r="J57" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K57" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G58" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G59" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G60" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H60" s="12"/>
+      <c r="J60" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K60" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G61" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G62" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H63" s="0"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G90" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H90" s="12"/>
+      <c r="J90" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K90" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L90" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G91" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G92" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G93" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H93" s="12"/>
+      <c r="J93" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K93" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G94" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G95" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G96" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H96" s="12"/>
+      <c r="J96" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K96" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L96" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G97" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G98" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G99" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H99" s="12"/>
+      <c r="J99" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K99" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G100" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G101" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G102" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H102" s="12"/>
+      <c r="J102" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K102" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G103" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G104" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G105" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H105" s="12"/>
+      <c r="J105" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K105" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L105" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G106" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G107" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G108" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H108" s="12"/>
+      <c r="J108" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K108" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G109" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G110" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G111" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H111" s="12"/>
+      <c r="J111" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K111" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G112" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G113" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G114" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H114" s="12"/>
+      <c r="J114" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K114" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G115" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G116" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H117" s="0"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G126" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H126" s="12"/>
+      <c r="J126" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K126" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G127" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G128" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G129" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H129" s="12"/>
+      <c r="J129" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K129" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L129" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G130" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G131" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G132" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H132" s="12"/>
+      <c r="J132" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K132" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L132" s="13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G133" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G134" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G135" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H135" s="12"/>
+      <c r="J135" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K135" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G136" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G137" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G138" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H138" s="12"/>
+      <c r="J138" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K138" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G139" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G140" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G141" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H141" s="12"/>
+      <c r="J141" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K141" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G142" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G143" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G144" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H144" s="12"/>
+      <c r="J144" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K144" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G145" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G146" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G147" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H147" s="12"/>
+      <c r="J147" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K147" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L147" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G148" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G149" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G150" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H150" s="12"/>
+      <c r="J150" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K150" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G151" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G152" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G153" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H153" s="12"/>
+      <c r="J153" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K153" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="L153" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G154" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G155" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G156" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H156" s="12"/>
+      <c r="J156" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="K156" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G157" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G158" s="7" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="L2" r:id="rId1" location="Namespace" display="http://www.tkltd.org/ontologies/datamodel#Namespace"/>
+    <hyperlink ref="L11" r:id="rId2" location="Domain" display="http://www.tkltd.org/ontologies/datamodel#Domain"/>
+    <hyperlink ref="L20" r:id="rId3" location="DomainEvent" display="http://www.tkltd.org/ontologies/datamodel#DomainEvent"/>
+    <hyperlink ref="L32" r:id="rId4" location="DomainParticipant" display="http://www.tkltd.org/ontologies/datamodel#DomainParticipant"/>
+    <hyperlink ref="L42" r:id="rId5" location="Attribute" display="http://www.tkltd.org/ontologies/datamodel#Attribute"/>
+    <hyperlink ref="L51" r:id="rId6" location="Class" display="http://www.tkltd.org/ontologies/datamodel#Class"/>
+    <hyperlink ref="L90" r:id="rId7" location="Attribute" display="http://www.tkltd.org/ontologies/datamodel#Attribute"/>
+    <hyperlink ref="L96" r:id="rId8" location="Class" display="http://www.tkltd.org/ontologies/datamodel#Class"/>
+    <hyperlink ref="L105" r:id="rId9" location="Model" display="http://www.tkltd.org/ontologies/datamodel#Model"/>
+    <hyperlink ref="L129" r:id="rId10" location="Domain" display="http://www.tkltd.org/ontologies/datamodel#Domain"/>
+    <hyperlink ref="L132" r:id="rId11" location="Relationship" display="http://www.tkltd.org/ontologies/datamodel#Relationship"/>
+    <hyperlink ref="L147" r:id="rId12" location="Attribute" display="http://www.tkltd.org/ontologies/datamodel#Attribute"/>
+    <hyperlink ref="L153" r:id="rId13" location="Class" display="http://www.tkltd.org/ontologies/datamodel#Class"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -694,11 +1781,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="29.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="29.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.84"/>
@@ -707,22 +1794,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>